<commit_message>
Actualizar USUARIOS.xlsx desde FITOASISTE
</commit_message>
<xml_diff>
--- a/USUARIOS.xlsx
+++ b/USUARIOS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,48 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>USR0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VIVIANA VILLA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>30233368</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VIVIANAVILLA</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>8811</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>vialviar@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ASESOR</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>

</xml_diff>